<commit_message>
Sum points, not ticks, for the standard sheet's Cultural and Career Used
Cultural Used and Career Used summed columns B and C, which hold the
'x' marks for which skills a culture or career offers. SUM ignores
text, so both always read 0 and their Left figures never went down.
They now sum the points columns I and J, matching Free Used (K) and
the d20 generator, which already had this right.

Regenerated examples/Mythras_Character_Sheet_Enhanced.xlsx.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/Mythras_Character_Sheet_Enhanced.xlsx
+++ b/examples/Mythras_Character_Sheet_Enhanced.xlsx
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="E9">
-        <f>SUM(B:B)</f>
+        <f>SUM(I:I)</f>
         <v/>
       </c>
       <c r="N9" s="3" t="inlineStr">
@@ -677,7 +677,7 @@
         </is>
       </c>
       <c r="E10">
-        <f>SUM(C:C)</f>
+        <f>SUM(J:J)</f>
         <v/>
       </c>
       <c r="N10" s="3" t="inlineStr">

</xml_diff>